<commit_message>
Week 02: answer-sheet notes and a how-to line in the lecture workbook
- Tutorial Answers .docx: say that the screenshots show the original
  solution's output and the notebooks print the same numbers to
  2 decimals; "Investigate the following:" and "profit of £8." as in
  the tutorial sheet
- 2 LP with Excel Solver.xlsx: cell A12 explains how to run Solver and
  gives the answer (x = 41.14, y = 10.29, profit £277.71); the model
  and Solver settings are unchanged

Text only: no notebook, formula or result changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vw4nh2eHzV8787MFDT43D7

[skip ci]
</commit_message>
<xml_diff>
--- a/content/Lectures/Semester 1/Week 02 - Linear Programming 1/2 Lecture Demos/2 LP with Excel Solver.xlsx
+++ b/content/Lectures/Semester 1/Week 02 - Linear Programming 1/2 Lecture Demos/2 LP with Excel Solver.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Product X</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>Y</t>
+  </si>
+  <si>
+    <t>Lecture example (slides 3–13). Data → Solver → Solve (Simplex LP, maximise F10). Answer: x = 41.14, y = 10.29, profit £277.71.</t>
   </si>
 </sst>
 </file>
@@ -433,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -539,6 +542,11 @@
       <c r="F10">
         <f>B10*B3+C10*C3</f>
         <v>277.71428571428567</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>